<commit_message>
fix: delete all workflow
</commit_message>
<xml_diff>
--- a/Docs/excel_phan_he_chuc_nang.xlsx
+++ b/Docs/excel_phan_he_chuc_nang.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lập Trình Mạng\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9A50A6-BC98-4581-9B2E-D29AB3EF7D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B096D2CA-851B-4CF3-AF66-568B81D37FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9180" yWindow="0" windowWidth="19725" windowHeight="16305" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh mục mô đun" sheetId="2" r:id="rId1"/>
@@ -499,9 +499,6 @@
     <t>Giám sát, cảnh báo cho sinh viên và ghi hình màn hình sinh viên</t>
   </si>
   <si>
-    <t>Đưa file đề bài xuống máy sinh viên</t>
-  </si>
-  <si>
     <t>Thu bài nộp của sinh viên về Server và thống kê</t>
   </si>
   <si>
@@ -514,9 +511,6 @@
     <t>Xem, xóa và kiểm soát file ghi hình do M4 tạo ra</t>
   </si>
   <si>
-    <t>M4 (file ghi hình), M8</t>
-  </si>
-  <si>
     <t>Tên module</t>
   </si>
   <si>
@@ -527,6 +521,12 @@
   </si>
   <si>
     <t>Danh Mục Module Hệ thống Quản lý &amp; Giám sát Máy tính Nội bộ Trường Đại học Kiến trúc Đà Nẵng</t>
+  </si>
+  <si>
+    <t>M4, M8</t>
+  </si>
+  <si>
+    <t>đẩy file về server</t>
   </si>
 </sst>
 </file>
@@ -596,13 +596,6 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -617,6 +610,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -822,191 +822,191 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="A1" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="2" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A3)</f>
         <v>1</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="4" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A4)</f>
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A5)</f>
         <v>2</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A6)</f>
         <v>2</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="C7" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D7" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A7)</f>
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="8">
+      <c r="C8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A8)</f>
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="4" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="8">
+      <c r="C9" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A9)</f>
         <v>3</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="4" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="8">
+      <c r="C10" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A10)</f>
         <v>6</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="4" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D11" s="8">
+      <c r="C11" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="5">
         <f>COUNTIF('Phân hệ chức năng'!$F$3:$F$30,A11)</f>
         <v>5</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>162</v>
+      <c r="E11" s="4" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -1033,814 +1033,814 @@
     <col min="9" max="9" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="E2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
+      <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
+      <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+      <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+      <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+      <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="7" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+      <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="7" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="4" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+      <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+      <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+      <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="7" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+      <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="7" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="4" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+      <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+      <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="7" t="s">
+      <c r="B17" s="7"/>
+      <c r="C17" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="4" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+      <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2" t="s">
+      <c r="B18" s="7"/>
+      <c r="C18" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="4" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+      <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="7" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="4" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+      <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="4" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+      <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2" t="s">
+      <c r="B21" s="7"/>
+      <c r="C21" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="I21" s="4" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+      <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="7" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I22" s="4" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+      <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="7" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="I23" s="4" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+      <c r="A24" s="3">
         <v>22</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="7" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+      <c r="A25" s="3">
         <v>23</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="7" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="I25" s="7" t="s">
+      <c r="I25" s="4" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+      <c r="A26" s="3">
         <v>24</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="4" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+      <c r="A27" s="3">
         <v>25</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H27" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+      <c r="A28" s="3">
         <v>26</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="7" t="s">
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="I28" s="4" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+      <c r="A29" s="3">
         <v>27</v>
       </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="7" t="s">
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I29" s="4" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+      <c r="A30" s="3">
         <v>28</v>
       </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="7" t="s">
+      <c r="B30" s="7"/>
+      <c r="C30" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="4" t="s">
         <v>146</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="C13:C14"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="B20:B25"/>
     <mergeCell ref="C21:C25"/>
     <mergeCell ref="B26:B30"/>
     <mergeCell ref="C27:C29"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="C13:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>